<commit_message>
chore(demo): regenerate demo artifacts across packages; finegray text
Demo outputs were rerun on 29 Sep 2026, so demo figures and tables
moved. This covers the PNGs, .xlsx and .dta files under codescan/,
datamap/, eplot/, finegray/, iivw/, psdash/ and tabtools/, and adds new
setools/demo/*.html pages (cci_se, cdp, migrations, pira, sustainedss,
setools_overview). The datamap demo outputs now report datamap_version
1.7.0 and show SD/mean at three significant digits.
datamap/demo/demo_datamap.do drops quality and missing(detail) from the
JSON example, and console_datamap_missing.md adds the missing-value
pattern table. Separately, finegray_cif.ado, finegray_cif.sthlp,
finegray/README.md and qa/test_finegray_user_text.do change the
finegray_cif user-facing text.
</commit_message>
<xml_diff>
--- a/iivw/demo/iivw_reporting_exports.xlsx
+++ b/iivw/demo/iivw_reporting_exports.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="261" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="261" uniqueCount="122">
   <si>
     <t>IIVW balance diagnostic</t>
   </si>
@@ -362,12 +362,6 @@
     <t>1.1064</t>
   </si>
   <si>
-    <t>-0.0068</t>
-  </si>
-  <si>
-    <t>1.0068</t>
-  </si>
-  <si>
     <t>SE</t>
   </si>
   <si>
@@ -22651,7 +22645,7 @@
         <v>107</v>
       </c>
       <c r="D3" s="1263" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="E3" s="1309" t="s">
         <v>80</v>
@@ -22668,10 +22662,10 @@
         <v>108</v>
       </c>
       <c r="D4" s="1208" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="E4" s="1310" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="5">
@@ -22685,10 +22679,10 @@
         <v>109</v>
       </c>
       <c r="D5" s="1211" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="E5" s="1311" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="6">
@@ -22702,10 +22696,10 @@
         <v>110</v>
       </c>
       <c r="D6" s="1214" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="E6" s="1312" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="7">
@@ -22784,7 +22778,7 @@
         <v>101</v>
       </c>
       <c r="C11" s="1228" t="s">
-        <v>115</v>
+        <v>1</v>
       </c>
       <c r="D11" s="1229" t="s">
         <v>1</v>
@@ -22801,7 +22795,7 @@
         <v>102</v>
       </c>
       <c r="C12" s="1231" t="s">
-        <v>116</v>
+        <v>1</v>
       </c>
       <c r="D12" s="1232" t="s">
         <v>1</v>

</xml_diff>